<commit_message>
Updated scraper and grading to work
</commit_message>
<xml_diff>
--- a/output/graded_history/user_scorecards/2026-02-22.xlsx
+++ b/output/graded_history/user_scorecards/2026-02-22.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,6 +27,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FF0000"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00008000"/>
     </font>
   </fonts>
   <fills count="2">
@@ -55,11 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -535,14 +545,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -591,11 +599,7 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -647,14 +651,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K4" t="n">
+        <v>7</v>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -703,14 +705,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -759,14 +759,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K6" t="n">
+        <v>6</v>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -815,14 +813,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -871,14 +867,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K8" t="n">
+        <v>8</v>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -927,14 +921,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K9" t="n">
+        <v>7</v>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -983,14 +975,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K10" t="n">
+        <v>15</v>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1039,14 +1029,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K11" t="n">
+        <v>29</v>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1095,14 +1083,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K12" t="n">
+        <v>17</v>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1151,14 +1137,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K13" t="n">
+        <v>41</v>
+      </c>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1207,14 +1191,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1263,14 +1245,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K15" t="n">
+        <v>25</v>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1319,14 +1299,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K16" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1375,14 +1353,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K17" t="n">
+        <v>7</v>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1431,14 +1407,12 @@
           <t>S Tier</t>
         </is>
       </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1487,14 +1461,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L19" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K19" t="n">
+        <v>3</v>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1543,14 +1515,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K20" t="n">
+        <v>16</v>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1599,14 +1569,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K21" t="n">
+        <v>5</v>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1655,14 +1623,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K22" t="n">
+        <v>13</v>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1711,14 +1677,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K23" t="n">
+        <v>9</v>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -1767,14 +1731,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K24" t="n">
+        <v>42</v>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1823,14 +1785,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1879,14 +1839,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L26" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K26" t="n">
+        <v>2</v>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -1935,11 +1893,7 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -1991,14 +1945,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L28" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K28" t="n">
+        <v>7</v>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2047,14 +1999,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K29" t="n">
+        <v>1</v>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2103,14 +2053,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L30" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2159,14 +2107,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L31" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K31" t="n">
+        <v>25</v>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2215,14 +2161,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L32" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K32" t="n">
+        <v>1</v>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2271,14 +2215,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L33" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -2327,14 +2269,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L34" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K34" t="n">
+        <v>11</v>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2383,14 +2323,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L35" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K35" t="n">
+        <v>15</v>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2439,11 +2377,7 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -2495,11 +2429,7 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -2551,14 +2481,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L38" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K38" t="n">
+        <v>7</v>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -2607,14 +2535,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L39" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K39" t="n">
+        <v>10</v>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2663,14 +2589,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L40" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K40" t="n">
+        <v>28</v>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2719,14 +2643,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L41" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K41" t="n">
+        <v>4</v>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2775,14 +2697,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K42" t="n">
+        <v>5</v>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2831,14 +2751,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L43" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K43" t="n">
+        <v>3</v>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2887,14 +2805,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L44" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K44" t="n">
+        <v>3</v>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -2943,14 +2859,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L45" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K45" t="n">
+        <v>13</v>
+      </c>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -2999,14 +2913,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K46" t="n">
+        <v>26</v>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3055,14 +2967,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K47" t="n">
+        <v>7</v>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3111,14 +3021,12 @@
           <t>A Tier</t>
         </is>
       </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K48" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3167,11 +3075,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -3223,14 +3127,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K50" t="n">
+        <v>1</v>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3279,14 +3181,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K51" t="n">
+        <v>9</v>
+      </c>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -3335,11 +3235,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -3391,11 +3287,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -3447,14 +3339,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K54" t="n">
+        <v>5</v>
+      </c>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -3503,11 +3393,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -3559,14 +3445,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K56" t="n">
+        <v>1</v>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3615,14 +3499,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K57" t="n">
+        <v>9</v>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3671,14 +3553,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K58" t="n">
+        <v>30</v>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -3727,14 +3607,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K59" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K59" t="n">
+        <v>6</v>
+      </c>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -3783,11 +3661,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K60" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -3839,14 +3713,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K61" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K61" t="n">
+        <v>9</v>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -3895,14 +3767,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K62" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K62" t="n">
+        <v>18</v>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -3951,14 +3821,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K63" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K63" t="n">
+        <v>26</v>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4007,14 +3875,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K64" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K64" t="n">
+        <v>24</v>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -4063,14 +3929,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K65" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K65" t="n">
+        <v>12</v>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4119,14 +3983,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K66" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K66" t="n">
+        <v>1</v>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4175,11 +4037,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K67" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K67" t="inlineStr"/>
       <c r="L67" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -4231,14 +4089,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K68" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K68" t="n">
+        <v>3</v>
+      </c>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4287,14 +4143,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K69" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4343,14 +4197,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K70" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K70" t="n">
+        <v>6</v>
+      </c>
+      <c r="L70" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4399,14 +4251,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K71" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K71" t="n">
+        <v>14</v>
+      </c>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -4455,11 +4305,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K72" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K72" t="inlineStr"/>
       <c r="L72" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -4511,14 +4357,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K73" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K73" t="n">
+        <v>15</v>
+      </c>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -4567,14 +4411,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K74" t="n">
+        <v>12</v>
+      </c>
+      <c r="L74" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4623,14 +4465,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K75" t="n">
+        <v>2</v>
+      </c>
+      <c r="L75" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4679,14 +4519,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K76" t="n">
+        <v>2</v>
+      </c>
+      <c r="L76" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4735,14 +4573,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K77" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K77" t="n">
+        <v>9</v>
+      </c>
+      <c r="L77" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4791,14 +4627,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K78" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K78" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -4847,14 +4681,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K79" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K79" t="n">
+        <v>5</v>
+      </c>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -4903,14 +4735,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K80" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K80" t="n">
+        <v>9</v>
+      </c>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -4959,14 +4789,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K81" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K81" t="n">
+        <v>1</v>
+      </c>
+      <c r="L81" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5015,14 +4843,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K82" t="n">
+        <v>6</v>
+      </c>
+      <c r="L82" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5071,14 +4897,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K83" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K83" t="n">
+        <v>14</v>
+      </c>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5127,14 +4951,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K84" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K84" t="n">
+        <v>6</v>
+      </c>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5183,14 +5005,12 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K85" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K85" t="n">
+        <v>3</v>
+      </c>
+      <c r="L85" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5239,11 +5059,7 @@
           <t>B Tier</t>
         </is>
       </c>
-      <c r="K86" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K86" t="inlineStr"/>
       <c r="L86" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -5295,14 +5111,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K87" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K87" t="n">
+        <v>6</v>
+      </c>
+      <c r="L87" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5351,14 +5165,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K88" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K88" t="n">
+        <v>22</v>
+      </c>
+      <c r="L88" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5407,14 +5219,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L89" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K89" t="n">
+        <v>2</v>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5463,11 +5273,7 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K90" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K90" t="inlineStr"/>
       <c r="L90" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -5519,14 +5325,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K91" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L91" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K91" t="n">
+        <v>10</v>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5575,14 +5379,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K92" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L92" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K92" t="n">
+        <v>7</v>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5631,14 +5433,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K93" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K93" t="n">
+        <v>2</v>
+      </c>
+      <c r="L93" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5687,14 +5487,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K94" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L94" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K94" t="n">
+        <v>4</v>
+      </c>
+      <c r="L94" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5743,14 +5541,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K95" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L95" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K95" t="n">
+        <v>29</v>
+      </c>
+      <c r="L95" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5799,14 +5595,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K96" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L96" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K96" t="n">
+        <v>24</v>
+      </c>
+      <c r="L96" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5855,14 +5649,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K97" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L97" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K97" t="n">
+        <v>4</v>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -5911,14 +5703,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K98" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L98" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K98" t="n">
+        <v>7</v>
+      </c>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -5967,14 +5757,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L99" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K99" t="n">
+        <v>5</v>
+      </c>
+      <c r="L99" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6023,14 +5811,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K100" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L100" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K100" t="n">
+        <v>7</v>
+      </c>
+      <c r="L100" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6079,14 +5865,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K101" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L101" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K101" t="n">
+        <v>14</v>
+      </c>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6135,14 +5919,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K102" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L102" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K102" t="n">
+        <v>4</v>
+      </c>
+      <c r="L102" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6191,14 +5973,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K103" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L103" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K103" t="n">
+        <v>15</v>
+      </c>
+      <c r="L103" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6247,14 +6027,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K104" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L104" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K104" t="n">
+        <v>1</v>
+      </c>
+      <c r="L104" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6303,14 +6081,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K105" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L105" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K105" t="n">
+        <v>6</v>
+      </c>
+      <c r="L105" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6359,14 +6135,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K106" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L106" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K106" t="n">
+        <v>2</v>
+      </c>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6415,14 +6189,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K107" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L107" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K107" t="n">
+        <v>12</v>
+      </c>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6471,11 +6243,7 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K108" t="inlineStr"/>
       <c r="L108" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -6527,14 +6295,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K109" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L109" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K109" t="n">
+        <v>2</v>
+      </c>
+      <c r="L109" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6583,14 +6349,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K110" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L110" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K110" t="n">
+        <v>8</v>
+      </c>
+      <c r="L110" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6639,14 +6403,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K111" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L111" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K111" t="n">
+        <v>20</v>
+      </c>
+      <c r="L111" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6695,14 +6457,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K112" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L112" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K112" t="n">
+        <v>4</v>
+      </c>
+      <c r="L112" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6751,14 +6511,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K113" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L113" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K113" t="n">
+        <v>2</v>
+      </c>
+      <c r="L113" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6807,14 +6565,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K114" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L114" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K114" t="n">
+        <v>28</v>
+      </c>
+      <c r="L114" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -6863,14 +6619,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L115" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K115" t="n">
+        <v>7</v>
+      </c>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6919,14 +6673,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K116" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L116" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K116" t="n">
+        <v>1</v>
+      </c>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -6975,14 +6727,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K117" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L117" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K117" t="n">
+        <v>8</v>
+      </c>
+      <c r="L117" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7031,14 +6781,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K118" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L118" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K118" t="n">
+        <v>4</v>
+      </c>
+      <c r="L118" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7087,14 +6835,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K119" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L119" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K119" t="n">
+        <v>3</v>
+      </c>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7143,11 +6889,7 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K120" t="inlineStr"/>
       <c r="L120" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -7199,14 +6941,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K121" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L121" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K121" t="n">
+        <v>8</v>
+      </c>
+      <c r="L121" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7255,11 +6995,7 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K122" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K122" t="inlineStr"/>
       <c r="L122" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -7311,14 +7047,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K123" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L123" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K123" t="n">
+        <v>5</v>
+      </c>
+      <c r="L123" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7367,14 +7101,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K124" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L124" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K124" t="n">
+        <v>2</v>
+      </c>
+      <c r="L124" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7423,14 +7155,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K125" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L125" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K125" t="n">
+        <v>18</v>
+      </c>
+      <c r="L125" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7479,14 +7209,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K126" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L126" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K126" t="n">
+        <v>3</v>
+      </c>
+      <c r="L126" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7535,14 +7263,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K127" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L127" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K127" t="n">
+        <v>5</v>
+      </c>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7591,14 +7317,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K128" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L128" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K128" t="n">
+        <v>5</v>
+      </c>
+      <c r="L128" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7647,14 +7371,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K129" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L129" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K129" t="n">
+        <v>25</v>
+      </c>
+      <c r="L129" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7703,14 +7425,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K130" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L130" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K130" t="n">
+        <v>9</v>
+      </c>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -7759,11 +7479,7 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K131" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K131" t="inlineStr"/>
       <c r="L131" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -7815,14 +7531,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K132" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L132" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K132" t="n">
+        <v>3</v>
+      </c>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7871,14 +7585,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K133" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L133" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K133" t="n">
+        <v>1</v>
+      </c>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7927,14 +7639,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K134" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L134" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K134" t="n">
+        <v>6</v>
+      </c>
+      <c r="L134" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -7983,14 +7693,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K135" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L135" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K135" t="n">
+        <v>1</v>
+      </c>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8039,14 +7747,12 @@
           <t>C Tier</t>
         </is>
       </c>
-      <c r="K136" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L136" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K136" t="n">
+        <v>20</v>
+      </c>
+      <c r="L136" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8095,11 +7801,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K137" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K137" t="inlineStr"/>
       <c r="L137" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -8151,14 +7853,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K138" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L138" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K138" t="n">
+        <v>15</v>
+      </c>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8207,14 +7907,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K139" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L139" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K139" t="n">
+        <v>7</v>
+      </c>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8263,14 +7961,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K140" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L140" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K140" t="n">
+        <v>5</v>
+      </c>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8319,14 +8015,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K141" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L141" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K141" t="n">
+        <v>22</v>
+      </c>
+      <c r="L141" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8375,14 +8069,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K142" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L142" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K142" t="n">
+        <v>25</v>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8431,14 +8123,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K143" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L143" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K143" t="n">
+        <v>21</v>
+      </c>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8487,14 +8177,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K144" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L144" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K144" t="n">
+        <v>5</v>
+      </c>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8543,14 +8231,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L145" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K145" t="n">
+        <v>2</v>
+      </c>
+      <c r="L145" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8599,11 +8285,7 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
+      <c r="K146" t="inlineStr"/>
       <c r="L146" t="inlineStr">
         <is>
           <t>Pending / Not Found</t>
@@ -8655,14 +8337,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K147" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L147" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K147" t="n">
+        <v>7</v>
+      </c>
+      <c r="L147" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8711,14 +8391,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L148" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K148" t="n">
+        <v>17</v>
+      </c>
+      <c r="L148" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8767,14 +8445,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K149" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K149" t="n">
+        <v>0</v>
+      </c>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8823,14 +8499,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K150" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K150" t="n">
+        <v>20</v>
+      </c>
+      <c r="L150" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8879,14 +8553,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K151" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L151" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K151" t="n">
+        <v>8</v>
+      </c>
+      <c r="L151" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -8935,14 +8607,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K152" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L152" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K152" t="n">
+        <v>20</v>
+      </c>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -8991,14 +8661,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K153" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L153" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K153" t="n">
+        <v>0</v>
+      </c>
+      <c r="L153" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -9047,14 +8715,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K154" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L154" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K154" t="n">
+        <v>25</v>
+      </c>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -9103,14 +8769,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K155" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L155" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K155" t="n">
+        <v>24</v>
+      </c>
+      <c r="L155" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -9159,14 +8823,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K156" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L156" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K156" t="n">
+        <v>3</v>
+      </c>
+      <c r="L156" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -9215,14 +8877,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K157" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L157" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K157" t="n">
+        <v>1</v>
+      </c>
+      <c r="L157" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>
@@ -9271,14 +8931,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K158" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L158" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K158" t="n">
+        <v>9</v>
+      </c>
+      <c r="L158" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -9327,14 +8985,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K159" t="n">
+        <v>28</v>
+      </c>
+      <c r="L159" s="2" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
     </row>
@@ -9383,14 +9039,12 @@
           <t>Pass</t>
         </is>
       </c>
-      <c r="K160" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="L160" t="inlineStr">
-        <is>
-          <t>Pending / Not Found</t>
+      <c r="K160" t="n">
+        <v>4</v>
+      </c>
+      <c r="L160" s="3" t="inlineStr">
+        <is>
+          <t>WIN</t>
         </is>
       </c>
     </row>

</xml_diff>